<commit_message>
Further changes pre-start of MCV2
</commit_message>
<xml_diff>
--- a/app/config/tables/MADTRIAL_INC/Forms/MADTRIAL_INC/MADTRIAL_INC.xlsx
+++ b/app/config/tables/MADTRIAL_INC/Forms/MADTRIAL_INC/MADTRIAL_INC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afisker\Documents\tablet\MADtrials2\MADtrial\app\config\tables\MADTRIAL_INC\Forms\MADTRIAL_INC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFFE6F06-97ED-425F-A0FE-DE3298648C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7E5E4E-5D4E-4A7A-B760-922CB714689C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="502">
   <si>
     <t>setting_name</t>
   </si>
@@ -1517,9 +1517,6 @@
     <t>A criança deve ter entre 9 méses e 5 anos de idade</t>
   </si>
   <si>
-    <t>data('PODEVAC')=='2'|| data('PODEINC')=='2'  || data('JAINC') == '1' || data('BRACOCRI') &lt;110 || data('TEMPERATURA')&gt;37.9 || data('VENAOVAS') == '2' ||  data('VENAOVAS2') == '2' || (data('SARVAC') == '1' &amp;&amp;  data('SARVAC2') == '1')||data('SARVAC2') == '1'</t>
-  </si>
-  <si>
     <t>Josemira</t>
   </si>
   <si>
@@ -1536,6 +1533,30 @@
   </si>
   <si>
     <t>A criança recebeu os seus vacinas do sarampo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if </t>
+  </si>
+  <si>
+    <t>childAGE</t>
+  </si>
+  <si>
+    <t>adate.diffInDays(data("DOB"),data("DATINC"))</t>
+  </si>
+  <si>
+    <t>calculates.childAGE &lt;453 || adate.hasUncertainty(data('DOB')) &amp;&amp; (date('IDADEANO') == '1' &amp;&amp; data('IDADEMES')&lt; '3' || data('IDADEMES')&lt; '15')</t>
+  </si>
+  <si>
+    <t>data('PODEVAC')=='2'|| data('PODEINC')=='2'  || data('JAINC') == '1' || data('BRACOCRI') &lt;110 || data('TEMPERATURA')&gt;37.9 || data('VENAOVAS') == '2' ||  data('VENAOVAS2') == '2' || (data('SARVAC') == '1' &amp;&amp;  data('SARVAC2') != '2')||data('SARVAC2') == '1'</t>
+  </si>
+  <si>
+    <t>data('SARVAC') == '1' &amp;&amp; calculates.childAGE &lt;453</t>
+  </si>
+  <si>
+    <t>The child is not yet 15 months and has already received MV1</t>
+  </si>
+  <si>
+    <t>A crianca ainda nao completou 15 meses e ja tomou VAS1</t>
   </si>
 </sst>
 </file>
@@ -1592,7 +1613,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1614,6 +1635,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1641,7 +1668,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1658,6 +1685,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Excel Built-in Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2052,7 +2080,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:R239"/>
+  <dimension ref="A1:R246"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.453125" bestFit="1" customWidth="1"/>
@@ -3283,437 +3311,423 @@
     </row>
     <row r="107" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B107" t="s">
+        <v>494</v>
+      </c>
+      <c r="C107" s="14" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="108" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B108" t="s">
         <v>55</v>
       </c>
-      <c r="C107" t="s">
+      <c r="C108" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="108" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D108" t="s">
+    <row r="109" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D109" t="s">
         <v>98</v>
       </c>
-      <c r="E108" t="s">
+      <c r="E109" t="s">
         <v>157</v>
       </c>
-      <c r="F108" t="s">
+      <c r="F109" t="s">
         <v>211</v>
       </c>
-      <c r="G108" t="s">
+      <c r="G109" t="s">
         <v>212</v>
       </c>
-      <c r="H108" t="s">
+      <c r="H109" t="s">
         <v>213</v>
       </c>
-      <c r="K108" t="s">
+      <c r="K109" t="s">
         <v>214</v>
       </c>
-      <c r="L108" t="s">
+      <c r="L109" t="s">
         <v>199</v>
       </c>
-      <c r="M108" t="s">
+      <c r="M109" t="s">
         <v>200</v>
-      </c>
-    </row>
-    <row r="109" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B109" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="110" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B110" t="s">
-        <v>55</v>
-      </c>
-      <c r="C110" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="111" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D111" t="s">
-        <v>98</v>
-      </c>
-      <c r="E111" t="s">
-        <v>157</v>
-      </c>
-      <c r="F111" t="s">
-        <v>215</v>
-      </c>
-      <c r="G111" t="s">
-        <v>208</v>
-      </c>
-      <c r="H111" t="s">
-        <v>216</v>
-      </c>
-      <c r="K111" t="s">
-        <v>210</v>
-      </c>
-      <c r="L111" t="s">
-        <v>199</v>
-      </c>
-      <c r="M111" t="s">
-        <v>200</v>
+        <v>73</v>
       </c>
     </row>
     <row r="112" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B112" t="s">
+        <v>55</v>
+      </c>
+      <c r="C112" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="113" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="D113" t="s">
+        <v>98</v>
+      </c>
+      <c r="E113" t="s">
+        <v>157</v>
+      </c>
+      <c r="F113" t="s">
+        <v>215</v>
+      </c>
+      <c r="G113" t="s">
+        <v>208</v>
+      </c>
+      <c r="H113" t="s">
+        <v>216</v>
+      </c>
+      <c r="K113" t="s">
+        <v>210</v>
+      </c>
+      <c r="L113" t="s">
+        <v>199</v>
+      </c>
+      <c r="M113" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="114" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B114" s="14" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="113" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B113" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="114" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B114" t="s">
-        <v>55</v>
-      </c>
-      <c r="C114" t="s">
-        <v>201</v>
-      </c>
-    </row>
     <row r="115" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="D115" t="s">
-        <v>217</v>
-      </c>
-      <c r="F115" t="s">
-        <v>218</v>
-      </c>
-      <c r="G115" t="s">
-        <v>219</v>
-      </c>
-      <c r="H115" t="s">
-        <v>220</v>
+      <c r="B115" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="116" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B116" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
     </row>
     <row r="117" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B117" t="s">
-        <v>40</v>
+        <v>55</v>
+      </c>
+      <c r="C117" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="118" spans="2:16" x14ac:dyDescent="0.35">
       <c r="D118" t="s">
-        <v>63</v>
+        <v>217</v>
       </c>
       <c r="F118" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="G118" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="H118" t="s">
-        <v>223</v>
-      </c>
-      <c r="K118" t="s">
-        <v>224</v>
-      </c>
-      <c r="L118" t="s">
-        <v>225</v>
-      </c>
-      <c r="M118" t="s">
-        <v>226</v>
-      </c>
-      <c r="N118" t="s">
-        <v>227</v>
-      </c>
-      <c r="O118" t="s">
-        <v>228</v>
-      </c>
-      <c r="P118" t="s">
-        <v>92</v>
+        <v>220</v>
       </c>
     </row>
     <row r="119" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="D119" t="s">
-        <v>78</v>
-      </c>
-      <c r="F119" t="s">
-        <v>229</v>
-      </c>
-      <c r="G119" t="s">
-        <v>230</v>
-      </c>
-      <c r="H119" t="s">
-        <v>231</v>
-      </c>
-      <c r="K119" t="s">
-        <v>232</v>
-      </c>
-      <c r="L119" t="s">
-        <v>233</v>
-      </c>
-      <c r="M119" t="s">
-        <v>234</v>
+      <c r="B119" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="120" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B120" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="121" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B121" t="s">
-        <v>40</v>
+      <c r="D121" t="s">
+        <v>63</v>
+      </c>
+      <c r="F121" t="s">
+        <v>221</v>
+      </c>
+      <c r="G121" t="s">
+        <v>222</v>
+      </c>
+      <c r="H121" t="s">
+        <v>223</v>
+      </c>
+      <c r="K121" t="s">
+        <v>224</v>
+      </c>
+      <c r="L121" t="s">
+        <v>225</v>
+      </c>
+      <c r="M121" t="s">
+        <v>226</v>
+      </c>
+      <c r="N121" t="s">
+        <v>227</v>
+      </c>
+      <c r="O121" t="s">
+        <v>228</v>
+      </c>
+      <c r="P121" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="122" spans="2:16" x14ac:dyDescent="0.35">
       <c r="D122" t="s">
-        <v>98</v>
-      </c>
-      <c r="E122" t="s">
-        <v>235</v>
+        <v>78</v>
       </c>
       <c r="F122" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="G122" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="H122" t="s">
-        <v>238</v>
+        <v>231</v>
+      </c>
+      <c r="K122" t="s">
+        <v>232</v>
+      </c>
+      <c r="L122" t="s">
+        <v>233</v>
+      </c>
+      <c r="M122" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="123" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B123" t="s">
-        <v>55</v>
-      </c>
-      <c r="C123" t="s">
-        <v>239</v>
+        <v>49</v>
       </c>
     </row>
     <row r="124" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="D124" t="s">
-        <v>46</v>
-      </c>
-      <c r="F124" t="s">
-        <v>240</v>
-      </c>
-      <c r="G124" t="s">
-        <v>241</v>
-      </c>
-      <c r="H124" t="s">
-        <v>242</v>
-      </c>
-      <c r="K124" t="s">
-        <v>243</v>
-      </c>
-      <c r="L124" t="s">
-        <v>143</v>
-      </c>
-      <c r="M124" t="s">
-        <v>144</v>
+      <c r="B124" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="125" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B125" t="s">
-        <v>73</v>
+      <c r="D125" t="s">
+        <v>98</v>
+      </c>
+      <c r="E125" t="s">
+        <v>235</v>
+      </c>
+      <c r="F125" t="s">
+        <v>236</v>
+      </c>
+      <c r="G125" t="s">
+        <v>237</v>
+      </c>
+      <c r="H125" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="126" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B126" t="s">
+        <v>55</v>
+      </c>
+      <c r="C126" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="127" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="D127" t="s">
+        <v>46</v>
+      </c>
+      <c r="F127" t="s">
+        <v>240</v>
+      </c>
+      <c r="G127" t="s">
+        <v>241</v>
+      </c>
+      <c r="H127" t="s">
+        <v>242</v>
+      </c>
+      <c r="K127" t="s">
+        <v>243</v>
+      </c>
+      <c r="L127" t="s">
+        <v>143</v>
+      </c>
+      <c r="M127" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="128" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B128" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="129" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B129" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="127" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B127" t="s">
+    <row r="130" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B130" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="128" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="D128" t="s">
+    <row r="131" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="D131" t="s">
         <v>98</v>
       </c>
-      <c r="E128" t="s">
+      <c r="E131" t="s">
         <v>244</v>
       </c>
-      <c r="F128" t="s">
+      <c r="F131" t="s">
         <v>245</v>
       </c>
-      <c r="G128" t="s">
+      <c r="G131" t="s">
         <v>246</v>
       </c>
-      <c r="H128" t="s">
+      <c r="H131" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="129" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D129" t="s">
+    <row r="132" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="D132" t="s">
         <v>98</v>
       </c>
-      <c r="E129" t="s">
+      <c r="E132" t="s">
         <v>244</v>
       </c>
-      <c r="F129" t="s">
+      <c r="F132" t="s">
         <v>248</v>
       </c>
-      <c r="G129" t="s">
+      <c r="G132" t="s">
         <v>249</v>
       </c>
-      <c r="H129" t="s">
+      <c r="H132" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="130" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D130" t="s">
+    <row r="133" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="D133" t="s">
         <v>98</v>
       </c>
-      <c r="E130" t="s">
+      <c r="E133" t="s">
         <v>244</v>
       </c>
-      <c r="F130" t="s">
+      <c r="F133" t="s">
         <v>251</v>
       </c>
-      <c r="G130" t="s">
+      <c r="G133" t="s">
         <v>252</v>
       </c>
-      <c r="H130" t="s">
+      <c r="H133" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="131" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B131" s="7" t="s">
+    <row r="134" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B134" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C131" s="7" t="s">
+      <c r="C134" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="D131" s="7"/>
-      <c r="E131" s="7"/>
-      <c r="F131" s="7"/>
-      <c r="G131" s="7"/>
-      <c r="H131" s="7"/>
-      <c r="I131" s="7"/>
-    </row>
-    <row r="132" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B132" s="7"/>
-      <c r="C132" s="7"/>
-      <c r="D132" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E132" s="7"/>
-      <c r="F132" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="G132" s="7"/>
-      <c r="H132" s="7"/>
-      <c r="I132" s="7" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="133" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B133" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C133" s="7"/>
-      <c r="D133" s="7"/>
-      <c r="E133" s="7"/>
-      <c r="F133" s="7"/>
-      <c r="G133" s="7"/>
-      <c r="H133" s="7"/>
-      <c r="I133" s="7"/>
-    </row>
-    <row r="134" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B134" s="7"/>
-      <c r="C134" s="7"/>
-      <c r="D134" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="D134" s="7"/>
       <c r="E134" s="7"/>
-      <c r="F134" s="7" t="s">
-        <v>255</v>
-      </c>
+      <c r="F134" s="7"/>
       <c r="G134" s="7"/>
       <c r="H134" s="7"/>
-      <c r="I134" s="7" t="s">
-        <v>257</v>
-      </c>
+      <c r="I134" s="7"/>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B135" s="7" t="s">
-        <v>73</v>
-      </c>
+      <c r="B135" s="7"/>
       <c r="C135" s="7"/>
-      <c r="D135" s="7"/>
+      <c r="D135" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="E135" s="7"/>
-      <c r="F135" s="7"/>
+      <c r="F135" s="7" t="s">
+        <v>255</v>
+      </c>
       <c r="G135" s="7"/>
       <c r="H135" s="7"/>
-      <c r="I135" s="7"/>
+      <c r="I135" s="7" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B136" t="s">
+      <c r="B136" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C136" s="7"/>
+      <c r="D136" s="7"/>
+      <c r="E136" s="7"/>
+      <c r="F136" s="7"/>
+      <c r="G136" s="7"/>
+      <c r="H136" s="7"/>
+      <c r="I136" s="7"/>
+    </row>
+    <row r="137" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B137" s="7"/>
+      <c r="C137" s="7"/>
+      <c r="D137" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E137" s="7"/>
+      <c r="F137" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="G137" s="7"/>
+      <c r="H137" s="7"/>
+      <c r="I137" s="7" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="138" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B138" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C138" s="7"/>
+      <c r="D138" s="7"/>
+      <c r="E138" s="7"/>
+      <c r="F138" s="7"/>
+      <c r="G138" s="7"/>
+      <c r="H138" s="7"/>
+      <c r="I138" s="7"/>
+    </row>
+    <row r="139" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B139" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="137" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B137" t="s">
+    <row r="140" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B140" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="138" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D138" t="s">
+    <row r="141" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="D141" t="s">
         <v>98</v>
       </c>
-      <c r="E138" t="s">
+      <c r="E141" t="s">
         <v>244</v>
       </c>
-      <c r="F138" t="s">
+      <c r="F141" t="s">
         <v>258</v>
       </c>
-      <c r="G138" t="s">
+      <c r="G141" t="s">
         <v>259</v>
       </c>
-      <c r="H138" t="s">
+      <c r="H141" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="139" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D139" t="s">
+    <row r="142" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="D142" t="s">
         <v>98</v>
       </c>
-      <c r="E139" t="s">
+      <c r="E142" t="s">
         <v>244</v>
       </c>
-      <c r="F139" t="s">
+      <c r="F142" t="s">
         <v>261</v>
       </c>
-      <c r="G139" t="s">
+      <c r="G142" t="s">
         <v>262</v>
       </c>
-      <c r="H139" t="s">
+      <c r="H142" t="s">
         <v>263</v>
-      </c>
-    </row>
-    <row r="140" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D140" t="s">
-        <v>98</v>
-      </c>
-      <c r="E140" t="s">
-        <v>244</v>
-      </c>
-      <c r="F140" t="s">
-        <v>264</v>
-      </c>
-      <c r="G140" t="s">
-        <v>265</v>
-      </c>
-      <c r="H140" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="141" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B141" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="142" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B142" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.35">
@@ -3724,223 +3738,226 @@
         <v>244</v>
       </c>
       <c r="F143" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="G143" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="H143" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D144" t="s">
-        <v>63</v>
-      </c>
-      <c r="F144" t="s">
-        <v>270</v>
-      </c>
-      <c r="G144" t="s">
-        <v>271</v>
-      </c>
-      <c r="H144" t="s">
-        <v>272</v>
+      <c r="B144" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="145" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B145" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="146" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="D146" t="s">
+        <v>98</v>
+      </c>
+      <c r="E146" t="s">
+        <v>244</v>
+      </c>
+      <c r="F146" t="s">
+        <v>267</v>
+      </c>
+      <c r="G146" t="s">
+        <v>268</v>
+      </c>
+      <c r="H146" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="147" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="D147" t="s">
+        <v>63</v>
+      </c>
+      <c r="F147" t="s">
+        <v>270</v>
+      </c>
+      <c r="G147" t="s">
+        <v>271</v>
+      </c>
+      <c r="H147" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="148" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B148" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="146" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B146" s="8" t="s">
+    <row r="149" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B149" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="147" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D147" s="8" t="s">
+    <row r="150" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D150" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="E147" s="8" t="s">
+      <c r="E150" s="8" t="s">
         <v>244</v>
       </c>
-      <c r="F147" s="8" t="s">
+      <c r="F150" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="G147" s="8" t="s">
+      <c r="G150" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="H147" s="8" t="s">
+      <c r="H150" s="8" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="148" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B148" s="8" t="s">
+    <row r="151" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B151" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C148" s="8" t="s">
+      <c r="C151" s="8" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="149" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D149" s="8" t="s">
+    <row r="152" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D152" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E149" s="8" t="s">
+      <c r="E152" s="8" t="s">
         <v>277</v>
       </c>
-      <c r="F149" s="8" t="s">
+      <c r="F152" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="G149" s="8" t="s">
+      <c r="G152" s="8" t="s">
         <v>279</v>
       </c>
-      <c r="H149" s="8" t="s">
+      <c r="H152" s="8" t="s">
         <v>280</v>
-      </c>
-    </row>
-    <row r="150" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B150" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C150" s="8" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="151" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D151" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="F151" s="8" t="s">
-        <v>282</v>
-      </c>
-      <c r="G151" s="8" t="s">
-        <v>283</v>
-      </c>
-      <c r="H151" s="8" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="152" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B152" s="8" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="153" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B153" s="8" t="s">
-        <v>73</v>
+        <v>55</v>
+      </c>
+      <c r="C153" s="8" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="154" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B154" s="8" t="s">
-        <v>49</v>
+      <c r="D154" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F154" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="G154" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="H154" s="8" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="155" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B155" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="156" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B156" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="157" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B157" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="158" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B158" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="156" spans="2:8" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D156" s="5" t="s">
+    <row r="159" spans="2:8" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D159" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="E156" s="5" t="s">
+      <c r="E159" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="F156" s="5" t="s">
+      <c r="F159" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="G156" s="5" t="s">
+      <c r="G159" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="H156" s="5" t="s">
+      <c r="H159" s="5" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="157" spans="2:8" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B157" s="5" t="s">
+    <row r="160" spans="2:8" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B160" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C157" s="5" t="s">
+      <c r="C160" s="5" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="158" spans="2:8" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D158" s="5" t="s">
+    <row r="161" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D161" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E158" s="5" t="s">
+      <c r="E161" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="F158" s="5" t="s">
+      <c r="F161" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="G158" s="5" t="s">
+      <c r="G161" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="H158" s="5" t="s">
+      <c r="H161" s="5" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="159" spans="2:8" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B159" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C159" s="5" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="160" spans="2:8" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D160" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F160" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="G160" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="H160" s="5" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="161" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B161" s="5" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="162" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B162" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C162" s="5" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="163" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D163" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F163" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="G163" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="H163" s="5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="164" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B164" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="163" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B163" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="164" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B164" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="165" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D165" t="s">
-        <v>217</v>
-      </c>
-      <c r="F165" t="s">
-        <v>294</v>
-      </c>
-      <c r="G165" t="s">
-        <v>295</v>
-      </c>
-      <c r="H165" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="166" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B166" t="s">
+    <row r="165" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B165" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="166" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B166" s="5" t="s">
         <v>49</v>
       </c>
     </row>
@@ -3951,265 +3968,265 @@
     </row>
     <row r="168" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D168" t="s">
-        <v>98</v>
-      </c>
-      <c r="E168" t="s">
-        <v>157</v>
+        <v>217</v>
       </c>
       <c r="F168" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="G168" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="H168" t="s">
-        <v>299</v>
-      </c>
-      <c r="K168" t="s">
-        <v>300</v>
-      </c>
-      <c r="L168" t="s">
-        <v>199</v>
-      </c>
-      <c r="M168" t="s">
-        <v>200</v>
+        <v>296</v>
       </c>
     </row>
     <row r="169" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B169" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="170" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B170" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="171" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D171" t="s">
+        <v>98</v>
+      </c>
+      <c r="E171" t="s">
+        <v>157</v>
+      </c>
+      <c r="F171" t="s">
+        <v>297</v>
+      </c>
+      <c r="G171" t="s">
+        <v>298</v>
+      </c>
+      <c r="H171" t="s">
+        <v>299</v>
+      </c>
+      <c r="K171" t="s">
+        <v>300</v>
+      </c>
+      <c r="L171" t="s">
+        <v>199</v>
+      </c>
+      <c r="M171" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="172" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B172" t="s">
         <v>55</v>
       </c>
-      <c r="C169" t="s">
+      <c r="C172" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="170" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D170" t="s">
+    <row r="173" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D173" t="s">
         <v>63</v>
       </c>
-      <c r="F170" t="s">
+      <c r="F173" t="s">
         <v>302</v>
       </c>
-      <c r="G170" t="s">
+      <c r="G173" t="s">
         <v>303</v>
       </c>
-      <c r="H170" t="s">
+      <c r="H173" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="171" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B171" t="s">
+    <row r="174" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B174" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="172" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D172" t="s">
+    <row r="175" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D175" t="s">
         <v>98</v>
       </c>
-      <c r="E172" t="s">
+      <c r="E175" t="s">
         <v>157</v>
       </c>
-      <c r="F172" t="s">
+      <c r="F175" t="s">
         <v>305</v>
       </c>
-      <c r="G172" t="s">
+      <c r="G175" t="s">
         <v>306</v>
       </c>
-      <c r="H172" t="s">
+      <c r="H175" t="s">
         <v>307</v>
       </c>
-      <c r="K172" t="s">
+      <c r="K175" t="s">
         <v>308</v>
       </c>
-      <c r="L172" t="s">
+      <c r="L175" t="s">
         <v>199</v>
       </c>
-      <c r="M172" t="s">
+      <c r="M175" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="173" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B173" t="s">
+    <row r="176" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B176" t="s">
         <v>55</v>
       </c>
-      <c r="C173" t="s">
+      <c r="C176" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="174" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D174" t="s">
+    <row r="177" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D177" t="s">
         <v>63</v>
       </c>
-      <c r="F174" t="s">
+      <c r="F177" t="s">
         <v>310</v>
       </c>
-      <c r="G174" t="s">
+      <c r="G177" t="s">
         <v>303</v>
       </c>
-      <c r="H174" t="s">
+      <c r="H177" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="175" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B175" t="s">
+    <row r="178" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B178" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="176" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D176" t="s">
+    <row r="179" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D179" t="s">
         <v>98</v>
       </c>
-      <c r="E176" t="s">
+      <c r="E179" t="s">
         <v>244</v>
       </c>
-      <c r="F176" t="s">
+      <c r="F179" t="s">
         <v>311</v>
       </c>
-      <c r="G176" t="s">
+      <c r="G179" t="s">
         <v>312</v>
       </c>
-      <c r="H176" t="s">
+      <c r="H179" t="s">
         <v>313</v>
       </c>
-      <c r="K176" t="s">
+      <c r="K179" t="s">
         <v>314</v>
       </c>
-      <c r="L176" t="s">
+      <c r="L179" t="s">
         <v>199</v>
       </c>
-      <c r="M176" t="s">
+      <c r="M179" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="177" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B177" t="s">
+    <row r="180" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B180" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="178" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B178" t="s">
+    <row r="181" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B181" t="s">
         <v>55</v>
       </c>
-      <c r="C178" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="179" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B179" t="s">
+      <c r="C181" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="182" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B182" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="180" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D180" t="s">
+    <row r="183" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D183" t="s">
         <v>41</v>
       </c>
-      <c r="F180" t="s">
+      <c r="F183" t="s">
         <v>315</v>
       </c>
-      <c r="I180">
+      <c r="I183">
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D181" t="s">
+    <row r="184" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D184" t="s">
         <v>156</v>
       </c>
-      <c r="G181" t="s">
+      <c r="G184" t="s">
         <v>316</v>
       </c>
-      <c r="H181" t="s">
+      <c r="H184" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="182" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B182" t="s">
-        <v>55</v>
-      </c>
-      <c r="C182" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="183" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D183" t="s">
-        <v>156</v>
-      </c>
-      <c r="G183" t="s">
-        <v>318</v>
-      </c>
-      <c r="H183" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="184" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B184" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="185" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="185" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B185" t="s">
         <v>55</v>
       </c>
       <c r="C185" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="186" spans="2:9" x14ac:dyDescent="0.35">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="186" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D186" t="s">
         <v>156</v>
       </c>
       <c r="G186" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H186" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="187" spans="2:9" x14ac:dyDescent="0.35">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="187" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B187" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="188" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="188" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B188" t="s">
         <v>55</v>
       </c>
       <c r="C188" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="189" spans="2:9" x14ac:dyDescent="0.35">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="189" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D189" t="s">
         <v>156</v>
       </c>
       <c r="G189" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="H189" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="190" spans="2:9" x14ac:dyDescent="0.35">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="190" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B190" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="191" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="191" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B191" t="s">
         <v>55</v>
       </c>
       <c r="C191" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="192" spans="2:9" x14ac:dyDescent="0.35">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="192" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D192" t="s">
         <v>156</v>
       </c>
       <c r="G192" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="H192" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="193" spans="2:8" x14ac:dyDescent="0.35">
@@ -4222,7 +4239,7 @@
         <v>55</v>
       </c>
       <c r="C194" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="195" spans="2:8" x14ac:dyDescent="0.35">
@@ -4230,10 +4247,10 @@
         <v>156</v>
       </c>
       <c r="G195" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H195" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="196" spans="2:8" x14ac:dyDescent="0.35">
@@ -4246,7 +4263,7 @@
         <v>55</v>
       </c>
       <c r="C197" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="198" spans="2:8" x14ac:dyDescent="0.35">
@@ -4254,10 +4271,10 @@
         <v>156</v>
       </c>
       <c r="G198" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="H198" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="199" spans="2:8" x14ac:dyDescent="0.35">
@@ -4270,7 +4287,7 @@
         <v>55</v>
       </c>
       <c r="C200" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
     </row>
     <row r="201" spans="2:8" x14ac:dyDescent="0.35">
@@ -4278,10 +4295,10 @@
         <v>156</v>
       </c>
       <c r="G201" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="H201" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
     </row>
     <row r="202" spans="2:8" x14ac:dyDescent="0.35">
@@ -4294,7 +4311,7 @@
         <v>55</v>
       </c>
       <c r="C203" t="s">
-        <v>492</v>
+        <v>334</v>
       </c>
     </row>
     <row r="204" spans="2:8" x14ac:dyDescent="0.35">
@@ -4302,10 +4319,10 @@
         <v>156</v>
       </c>
       <c r="G204" t="s">
-        <v>493</v>
+        <v>335</v>
       </c>
       <c r="H204" t="s">
-        <v>494</v>
+        <v>336</v>
       </c>
     </row>
     <row r="205" spans="2:8" x14ac:dyDescent="0.35">
@@ -4318,7 +4335,7 @@
         <v>55</v>
       </c>
       <c r="C206" t="s">
-        <v>337</v>
+        <v>491</v>
       </c>
     </row>
     <row r="207" spans="2:8" x14ac:dyDescent="0.35">
@@ -4326,10 +4343,10 @@
         <v>156</v>
       </c>
       <c r="G207" t="s">
-        <v>338</v>
+        <v>492</v>
       </c>
       <c r="H207" t="s">
-        <v>339</v>
+        <v>493</v>
       </c>
     </row>
     <row r="208" spans="2:8" x14ac:dyDescent="0.35">
@@ -4337,323 +4354,371 @@
         <v>73</v>
       </c>
     </row>
-    <row r="209" spans="2:17" x14ac:dyDescent="0.35">
+    <row r="209" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B209" t="s">
+        <v>55</v>
+      </c>
+      <c r="C209" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="210" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D210" t="s">
+        <v>156</v>
+      </c>
+      <c r="G210" t="s">
+        <v>338</v>
+      </c>
+      <c r="H210" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="211" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B211" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="213" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B213" t="s">
+        <v>55</v>
+      </c>
+      <c r="C213" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="214" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D214" t="s">
+        <v>156</v>
+      </c>
+      <c r="G214" t="s">
+        <v>500</v>
+      </c>
+      <c r="H214" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="215" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B215" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="216" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B216" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="210" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B210" t="s">
+    <row r="217" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B217" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="211" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B211" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="212" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D212" t="s">
-        <v>78</v>
-      </c>
-      <c r="F212" t="s">
-        <v>340</v>
-      </c>
-      <c r="G212" t="s">
-        <v>341</v>
-      </c>
-      <c r="H212" t="s">
-        <v>342</v>
-      </c>
-      <c r="K212" t="s">
-        <v>343</v>
-      </c>
-      <c r="L212" t="s">
-        <v>344</v>
-      </c>
-      <c r="M212" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="213" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D213" t="s">
-        <v>78</v>
-      </c>
-      <c r="F213" t="s">
-        <v>346</v>
-      </c>
-      <c r="G213" t="s">
-        <v>347</v>
-      </c>
-      <c r="H213" t="s">
-        <v>348</v>
-      </c>
-      <c r="K213" t="s">
-        <v>349</v>
-      </c>
-      <c r="L213" t="s">
-        <v>350</v>
-      </c>
-      <c r="M213" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="214" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D214" t="s">
-        <v>41</v>
-      </c>
-      <c r="F214" t="s">
-        <v>352</v>
-      </c>
-      <c r="I214" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="215" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D215" t="s">
-        <v>156</v>
-      </c>
-      <c r="G215" t="s">
-        <v>354</v>
-      </c>
-      <c r="H215" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="216" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D216" t="s">
-        <v>41</v>
-      </c>
-      <c r="F216" t="s">
-        <v>315</v>
-      </c>
-      <c r="I216">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="217" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B217" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="218" spans="2:17" x14ac:dyDescent="0.35">
+    <row r="218" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B218" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="219" spans="2:17" x14ac:dyDescent="0.35">
+    <row r="219" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D219" t="s">
+        <v>78</v>
+      </c>
+      <c r="F219" t="s">
+        <v>340</v>
+      </c>
+      <c r="G219" t="s">
+        <v>341</v>
+      </c>
+      <c r="H219" t="s">
+        <v>342</v>
+      </c>
+      <c r="K219" t="s">
+        <v>343</v>
+      </c>
+      <c r="L219" t="s">
+        <v>344</v>
+      </c>
+      <c r="M219" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="220" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D220" t="s">
+        <v>78</v>
+      </c>
+      <c r="F220" t="s">
+        <v>346</v>
+      </c>
+      <c r="G220" t="s">
+        <v>347</v>
+      </c>
+      <c r="H220" t="s">
+        <v>348</v>
+      </c>
+      <c r="K220" t="s">
+        <v>349</v>
+      </c>
+      <c r="L220" t="s">
+        <v>350</v>
+      </c>
+      <c r="M220" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="221" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D221" t="s">
         <v>41</v>
       </c>
-      <c r="F219" t="s">
+      <c r="F221" t="s">
+        <v>352</v>
+      </c>
+      <c r="I221" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="222" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D222" t="s">
+        <v>156</v>
+      </c>
+      <c r="G222" t="s">
+        <v>354</v>
+      </c>
+      <c r="H222" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="223" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D223" t="s">
+        <v>41</v>
+      </c>
+      <c r="F223" t="s">
+        <v>315</v>
+      </c>
+      <c r="I223">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B224" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="225" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="B225" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="226" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="D226" t="s">
+        <v>41</v>
+      </c>
+      <c r="F226" t="s">
         <v>356</v>
       </c>
-      <c r="I219" t="s">
+      <c r="I226" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="220" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D220" t="s">
+    <row r="227" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="D227" t="s">
         <v>46</v>
       </c>
-      <c r="F220" t="s">
+      <c r="F227" t="s">
         <v>356</v>
       </c>
-      <c r="G220" t="s">
+      <c r="G227" t="s">
         <v>358</v>
       </c>
-      <c r="H220" t="s">
+      <c r="H227" t="s">
         <v>359</v>
       </c>
-      <c r="Q220" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="221" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D221" t="s">
+      <c r="Q227" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="D228" t="s">
         <v>360</v>
       </c>
-      <c r="F221" t="s">
+      <c r="F228" t="s">
         <v>361</v>
       </c>
-      <c r="G221" t="s">
+      <c r="G228" t="s">
         <v>362</v>
       </c>
-      <c r="H221" t="s">
+      <c r="H228" t="s">
         <v>363</v>
       </c>
-      <c r="K221" t="s">
+      <c r="K228" t="s">
         <v>364</v>
       </c>
-      <c r="L221" t="s">
+      <c r="L228" t="s">
         <v>199</v>
       </c>
-      <c r="M221" t="s">
+      <c r="M228" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="222" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D222" t="s">
+    <row r="229" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="D229" t="s">
         <v>41</v>
       </c>
-      <c r="F222" t="s">
+      <c r="F229" t="s">
         <v>365</v>
       </c>
-      <c r="I222" t="s">
+      <c r="I229" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="223" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D223" t="s">
+    <row r="230" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="D230" t="s">
         <v>78</v>
       </c>
-      <c r="F223" t="s">
+      <c r="F230" t="s">
         <v>367</v>
       </c>
-      <c r="G223" t="s">
+      <c r="G230" t="s">
         <v>368</v>
       </c>
-      <c r="H223" t="s">
+      <c r="H230" t="s">
         <v>369</v>
       </c>
-      <c r="K223" t="s">
+      <c r="K230" t="s">
         <v>370</v>
       </c>
-      <c r="L223" t="s">
+      <c r="L230" t="s">
         <v>371</v>
       </c>
-      <c r="M223" t="s">
+      <c r="M230" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="224" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="D224" t="s">
+    <row r="231" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="D231" t="s">
         <v>41</v>
       </c>
-      <c r="F224" t="s">
+      <c r="F231" t="s">
         <v>373</v>
       </c>
-      <c r="I224" t="s">
+      <c r="I231" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="225" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D225" t="s">
+    <row r="232" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="D232" t="s">
         <v>156</v>
       </c>
-      <c r="G225" t="s">
+      <c r="G232" t="s">
         <v>375</v>
       </c>
-      <c r="H225" t="s">
+      <c r="H232" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="226" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B226" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="227" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B227" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="228" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B228" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="229" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D229" t="s">
-        <v>106</v>
-      </c>
-      <c r="E229" t="s">
-        <v>377</v>
-      </c>
-      <c r="F229" t="s">
-        <v>378</v>
-      </c>
-      <c r="G229" t="s">
-        <v>379</v>
-      </c>
-      <c r="H229" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="230" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B230" t="s">
-        <v>55</v>
-      </c>
-      <c r="C230" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="231" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D231" t="s">
-        <v>106</v>
-      </c>
-      <c r="E231" t="s">
-        <v>382</v>
-      </c>
-      <c r="F231" t="s">
-        <v>383</v>
-      </c>
-      <c r="G231" t="s">
-        <v>384</v>
-      </c>
-      <c r="H231" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="232" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B232" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="233" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="233" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B233" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="234" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="234" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B234" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="235" spans="2:9" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="235" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B235" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="236" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="236" spans="2:17" x14ac:dyDescent="0.35">
       <c r="D236" t="s">
+        <v>106</v>
+      </c>
+      <c r="E236" t="s">
+        <v>377</v>
+      </c>
+      <c r="F236" t="s">
+        <v>378</v>
+      </c>
+      <c r="G236" t="s">
+        <v>379</v>
+      </c>
+      <c r="H236" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="237" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="B237" t="s">
+        <v>55</v>
+      </c>
+      <c r="C237" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="238" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="D238" t="s">
+        <v>106</v>
+      </c>
+      <c r="E238" t="s">
+        <v>382</v>
+      </c>
+      <c r="F238" t="s">
+        <v>383</v>
+      </c>
+      <c r="G238" t="s">
+        <v>384</v>
+      </c>
+      <c r="H238" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="239" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="B239" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="240" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="B240" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="241" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B241" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="242" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B242" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="243" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="D243" t="s">
         <v>156</v>
       </c>
-      <c r="G236" t="s">
+      <c r="G243" t="s">
         <v>386</v>
       </c>
-      <c r="H236" t="s">
+      <c r="H243" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="237" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="D237" t="s">
+    <row r="244" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="D244" t="s">
         <v>41</v>
       </c>
-      <c r="F237" t="s">
+      <c r="F244" t="s">
         <v>315</v>
       </c>
-      <c r="I237">
+      <c r="I244">
         <v>2</v>
       </c>
     </row>
-    <row r="238" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B238" t="s">
+    <row r="245" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B245" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="239" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B239" t="s">
+    <row r="246" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B246" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4912,10 +4977,10 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D16" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E16" t="s">
         <v>410</v>
@@ -4936,7 +5001,7 @@
         <v>406</v>
       </c>
       <c r="E17" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -4978,10 +5043,10 @@
         <v>5</v>
       </c>
       <c r="C20" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D20" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -4993,10 +5058,10 @@
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D21" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -5809,7 +5874,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.7265625" bestFit="1" customWidth="1"/>
@@ -5822,6 +5887,14 @@
       </c>
       <c r="B1" s="11" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>495</v>
+      </c>
+      <c r="B2" t="s">
+        <v>496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>